<commit_message>
Update AIP retail petrol prices
</commit_message>
<xml_diff>
--- a/data/petrol_weekly_prices.xlsx
+++ b/data/petrol_weekly_prices.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2168,6 +2168,38 @@
         <v>207.6</v>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="1" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B55" s="1" t="n">
+        <v>46278</v>
+      </c>
+      <c r="C55" t="n">
+        <v>209.8</v>
+      </c>
+      <c r="D55" t="n">
+        <v>218.6</v>
+      </c>
+      <c r="E55" t="n">
+        <v>209.6</v>
+      </c>
+      <c r="F55" t="n">
+        <v>211.2</v>
+      </c>
+      <c r="G55" t="n">
+        <v>206.5</v>
+      </c>
+      <c r="H55" t="n">
+        <v>209.9</v>
+      </c>
+      <c r="I55" t="n">
+        <v>218.3</v>
+      </c>
+      <c r="J55" t="n">
+        <v>214.7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>